<commit_message>
A lot of things
</commit_message>
<xml_diff>
--- a/services/backend/uploads/datos_escroto.xlsx
+++ b/services/backend/uploads/datos_escroto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Documents\INGERNIERIA-INFORMATICA\4-CARRERA\MATERIAS\TFG\Proyecto_simple\services\backend\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3AC7E7E-FA89-4070-B435-09AB5EA87D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926F5919-0803-4EA0-A8D9-8F4369F465C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2420,10 +2420,10 @@
     <t>prioridad</t>
   </si>
   <si>
-    <t>OTHER</t>
-  </si>
-  <si>
     <t>NONE</t>
+  </si>
+  <si>
+    <t>ESCROTO</t>
   </si>
 </sst>
 </file>
@@ -2431,7 +2431,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -2464,7 +2464,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2907,13 +2907,13 @@
         <v>29</v>
       </c>
       <c r="V2" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
@@ -2975,13 +2975,13 @@
         <v>35</v>
       </c>
       <c r="V3" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
@@ -3043,13 +3043,13 @@
         <v>39</v>
       </c>
       <c r="V4" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W4" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X4" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
@@ -3111,13 +3111,13 @@
         <v>29</v>
       </c>
       <c r="V5" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W5" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X5" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
@@ -3176,13 +3176,13 @@
         <v>46</v>
       </c>
       <c r="V6" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.3">
@@ -3244,13 +3244,13 @@
         <v>50</v>
       </c>
       <c r="V7" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W7" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X7" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
@@ -3312,13 +3312,13 @@
         <v>29</v>
       </c>
       <c r="V8" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W8" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X8" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
@@ -3380,13 +3380,13 @@
         <v>58</v>
       </c>
       <c r="V9" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W9" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X9" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.3">
@@ -3448,13 +3448,13 @@
         <v>63</v>
       </c>
       <c r="V10" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W10" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X10" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.3">
@@ -3516,13 +3516,13 @@
         <v>68</v>
       </c>
       <c r="V11" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W11" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X11" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
@@ -3584,13 +3584,13 @@
         <v>73</v>
       </c>
       <c r="V12" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W12" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X12" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
@@ -3652,13 +3652,13 @@
         <v>29</v>
       </c>
       <c r="V13" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W13" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X13" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
@@ -3720,13 +3720,13 @@
         <v>81</v>
       </c>
       <c r="V14" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W14" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X14" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
@@ -3788,13 +3788,13 @@
         <v>84</v>
       </c>
       <c r="V15" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
@@ -3856,13 +3856,13 @@
         <v>88</v>
       </c>
       <c r="V16" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W16" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X16" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.3">
@@ -3924,13 +3924,13 @@
         <v>29</v>
       </c>
       <c r="V17" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W17" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X17" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.3">
@@ -3992,13 +3992,13 @@
         <v>35</v>
       </c>
       <c r="V18" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W18" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X18" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.3">
@@ -4060,13 +4060,13 @@
         <v>101</v>
       </c>
       <c r="V19" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W19" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X19" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.3">
@@ -4128,13 +4128,13 @@
         <v>29</v>
       </c>
       <c r="V20" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W20" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X20" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
@@ -4196,13 +4196,13 @@
         <v>108</v>
       </c>
       <c r="V21" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W21" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X21" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
@@ -4264,13 +4264,13 @@
         <v>112</v>
       </c>
       <c r="V22" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W22" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X22" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
@@ -4332,13 +4332,13 @@
         <v>116</v>
       </c>
       <c r="V23" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W23" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X23" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
@@ -4397,13 +4397,13 @@
         <v>122</v>
       </c>
       <c r="V24" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W24" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X24" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
@@ -4462,13 +4462,13 @@
         <v>125</v>
       </c>
       <c r="V25" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W25" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X25" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
@@ -4530,13 +4530,13 @@
         <v>81</v>
       </c>
       <c r="V26" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W26" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X26" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
@@ -4598,13 +4598,13 @@
         <v>134</v>
       </c>
       <c r="V27" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W27" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X27" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.3">
@@ -4666,13 +4666,13 @@
         <v>29</v>
       </c>
       <c r="V28" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W28" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X28" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.3">
@@ -4734,13 +4734,13 @@
         <v>141</v>
       </c>
       <c r="V29" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W29" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X29" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.3">
@@ -4802,13 +4802,13 @@
         <v>29</v>
       </c>
       <c r="V30" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W30" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X30" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
@@ -4870,13 +4870,13 @@
         <v>29</v>
       </c>
       <c r="V31" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W31" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X31" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
@@ -4938,13 +4938,13 @@
         <v>151</v>
       </c>
       <c r="V32" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W32" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X32" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.3">
@@ -5003,13 +5003,13 @@
         <v>154</v>
       </c>
       <c r="V33" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W33" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X33" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
@@ -5071,13 +5071,13 @@
         <v>159</v>
       </c>
       <c r="V34" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W34" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X34" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.3">
@@ -5139,13 +5139,13 @@
         <v>163</v>
       </c>
       <c r="V35" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W35" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X35" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.3">
@@ -5207,13 +5207,13 @@
         <v>29</v>
       </c>
       <c r="V36" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W36" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X36" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.3">
@@ -5275,13 +5275,13 @@
         <v>112</v>
       </c>
       <c r="V37" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W37" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X37" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.3">
@@ -5343,13 +5343,13 @@
         <v>174</v>
       </c>
       <c r="V38" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W38" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X38" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.3">
@@ -5411,13 +5411,13 @@
         <v>178</v>
       </c>
       <c r="V39" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W39" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X39" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.3">
@@ -5476,13 +5476,13 @@
         <v>182</v>
       </c>
       <c r="V40" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W40" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X40" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.3">
@@ -5544,13 +5544,13 @@
         <v>29</v>
       </c>
       <c r="V41" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W41" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X41" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
@@ -5612,13 +5612,13 @@
         <v>191</v>
       </c>
       <c r="V42" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W42" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X42" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
@@ -5680,13 +5680,13 @@
         <v>29</v>
       </c>
       <c r="V43" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W43" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X43" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
@@ -5748,13 +5748,13 @@
         <v>199</v>
       </c>
       <c r="V44" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W44" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X44" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
@@ -5816,13 +5816,13 @@
         <v>202</v>
       </c>
       <c r="V45" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W45" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X45" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
@@ -5884,13 +5884,13 @@
         <v>207</v>
       </c>
       <c r="V46" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W46" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X46" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.3">
@@ -5952,13 +5952,13 @@
         <v>212</v>
       </c>
       <c r="V47" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W47" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X47" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.3">
@@ -6023,13 +6023,13 @@
         <v>218</v>
       </c>
       <c r="V48" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W48" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X48" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="49" spans="1:24" x14ac:dyDescent="0.3">
@@ -6088,13 +6088,13 @@
         <v>221</v>
       </c>
       <c r="V49" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W49" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X49" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="50" spans="1:24" x14ac:dyDescent="0.3">
@@ -6156,13 +6156,13 @@
         <v>226</v>
       </c>
       <c r="V50" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W50" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X50" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="51" spans="1:24" x14ac:dyDescent="0.3">
@@ -6224,13 +6224,13 @@
         <v>230</v>
       </c>
       <c r="V51" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W51" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X51" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="52" spans="1:24" x14ac:dyDescent="0.3">
@@ -6292,13 +6292,13 @@
         <v>235</v>
       </c>
       <c r="V52" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W52" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X52" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="53" spans="1:24" x14ac:dyDescent="0.3">
@@ -6360,13 +6360,13 @@
         <v>240</v>
       </c>
       <c r="V53" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W53" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X53" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="54" spans="1:24" x14ac:dyDescent="0.3">
@@ -6428,13 +6428,13 @@
         <v>246</v>
       </c>
       <c r="V54" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W54" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X54" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="55" spans="1:24" x14ac:dyDescent="0.3">
@@ -6493,13 +6493,13 @@
         <v>249</v>
       </c>
       <c r="V55" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W55" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X55" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="56" spans="1:24" x14ac:dyDescent="0.3">
@@ -6561,13 +6561,13 @@
         <v>207</v>
       </c>
       <c r="V56" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W56" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X56" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="57" spans="1:24" x14ac:dyDescent="0.3">
@@ -6629,13 +6629,13 @@
         <v>257</v>
       </c>
       <c r="V57" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W57" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X57" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="58" spans="1:24" x14ac:dyDescent="0.3">
@@ -6697,13 +6697,13 @@
         <v>263</v>
       </c>
       <c r="V58" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W58" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X58" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="59" spans="1:24" x14ac:dyDescent="0.3">
@@ -6765,13 +6765,13 @@
         <v>29</v>
       </c>
       <c r="V59" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W59" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X59" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="60" spans="1:24" x14ac:dyDescent="0.3">
@@ -6833,13 +6833,13 @@
         <v>29</v>
       </c>
       <c r="V60" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W60" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X60" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="61" spans="1:24" x14ac:dyDescent="0.3">
@@ -6901,13 +6901,13 @@
         <v>273</v>
       </c>
       <c r="V61" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W61" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X61" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="62" spans="1:24" x14ac:dyDescent="0.3">
@@ -6969,13 +6969,13 @@
         <v>278</v>
       </c>
       <c r="V62" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W62" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X62" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="63" spans="1:24" x14ac:dyDescent="0.3">
@@ -7037,13 +7037,13 @@
         <v>112</v>
       </c>
       <c r="V63" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W63" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X63" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="64" spans="1:24" x14ac:dyDescent="0.3">
@@ -7105,13 +7105,13 @@
         <v>287</v>
       </c>
       <c r="V64" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W64" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X64" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="65" spans="1:24" x14ac:dyDescent="0.3">
@@ -7173,13 +7173,13 @@
         <v>292</v>
       </c>
       <c r="V65" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W65" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X65" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="66" spans="1:24" x14ac:dyDescent="0.3">
@@ -7238,13 +7238,13 @@
         <v>294</v>
       </c>
       <c r="V66" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W66" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X66" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="67" spans="1:24" x14ac:dyDescent="0.3">
@@ -7306,13 +7306,13 @@
         <v>300</v>
       </c>
       <c r="V67" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W67" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X67" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="68" spans="1:24" x14ac:dyDescent="0.3">
@@ -7374,13 +7374,13 @@
         <v>305</v>
       </c>
       <c r="V68" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W68" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X68" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="69" spans="1:24" x14ac:dyDescent="0.3">
@@ -7442,13 +7442,13 @@
         <v>309</v>
       </c>
       <c r="V69" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W69" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X69" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="70" spans="1:24" x14ac:dyDescent="0.3">
@@ -7510,13 +7510,13 @@
         <v>29</v>
       </c>
       <c r="V70" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W70" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X70" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="71" spans="1:24" x14ac:dyDescent="0.3">
@@ -7578,13 +7578,13 @@
         <v>29</v>
       </c>
       <c r="V71" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W71" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X71" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="72" spans="1:24" x14ac:dyDescent="0.3">
@@ -7646,13 +7646,13 @@
         <v>29</v>
       </c>
       <c r="V72" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W72" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X72" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="73" spans="1:24" x14ac:dyDescent="0.3">
@@ -7714,13 +7714,13 @@
         <v>323</v>
       </c>
       <c r="V73" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W73" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X73" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="74" spans="1:24" x14ac:dyDescent="0.3">
@@ -7782,13 +7782,13 @@
         <v>29</v>
       </c>
       <c r="V74" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W74" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X74" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="75" spans="1:24" x14ac:dyDescent="0.3">
@@ -7850,13 +7850,13 @@
         <v>29</v>
       </c>
       <c r="V75" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W75" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X75" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="76" spans="1:24" x14ac:dyDescent="0.3">
@@ -7918,13 +7918,13 @@
         <v>29</v>
       </c>
       <c r="V76" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W76" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X76" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="77" spans="1:24" x14ac:dyDescent="0.3">
@@ -7986,13 +7986,13 @@
         <v>336</v>
       </c>
       <c r="V77" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W77" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X77" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="78" spans="1:24" x14ac:dyDescent="0.3">
@@ -8054,13 +8054,13 @@
         <v>340</v>
       </c>
       <c r="V78" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W78" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X78" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="79" spans="1:24" x14ac:dyDescent="0.3">
@@ -8119,13 +8119,13 @@
         <v>342</v>
       </c>
       <c r="V79" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W79" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X79" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="80" spans="1:24" x14ac:dyDescent="0.3">
@@ -8187,13 +8187,13 @@
         <v>29</v>
       </c>
       <c r="V80" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W80" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X80" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="81" spans="1:24" x14ac:dyDescent="0.3">
@@ -8255,13 +8255,13 @@
         <v>348</v>
       </c>
       <c r="V81" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W81" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X81" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="82" spans="1:24" x14ac:dyDescent="0.3">
@@ -8323,13 +8323,13 @@
         <v>352</v>
       </c>
       <c r="V82" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W82" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X82" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="83" spans="1:24" x14ac:dyDescent="0.3">
@@ -8388,13 +8388,13 @@
         <v>355</v>
       </c>
       <c r="V83" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W83" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X83" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="84" spans="1:24" x14ac:dyDescent="0.3">
@@ -8456,13 +8456,13 @@
         <v>360</v>
       </c>
       <c r="V84" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W84" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X84" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="85" spans="1:24" x14ac:dyDescent="0.3">
@@ -8521,13 +8521,13 @@
         <v>362</v>
       </c>
       <c r="V85" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W85" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X85" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="86" spans="1:24" x14ac:dyDescent="0.3">
@@ -8589,13 +8589,13 @@
         <v>367</v>
       </c>
       <c r="V86" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W86" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X86" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="87" spans="1:24" x14ac:dyDescent="0.3">
@@ -8657,13 +8657,13 @@
         <v>372</v>
       </c>
       <c r="V87" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W87" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X87" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="88" spans="1:24" x14ac:dyDescent="0.3">
@@ -8725,13 +8725,13 @@
         <v>377</v>
       </c>
       <c r="V88" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W88" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X88" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="89" spans="1:24" x14ac:dyDescent="0.3">
@@ -8793,13 +8793,13 @@
         <v>158</v>
       </c>
       <c r="V89" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W89" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X89" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="90" spans="1:24" x14ac:dyDescent="0.3">
@@ -8861,13 +8861,13 @@
         <v>386</v>
       </c>
       <c r="V90" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W90" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X90" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="91" spans="1:24" x14ac:dyDescent="0.3">
@@ -8929,13 +8929,13 @@
         <v>391</v>
       </c>
       <c r="V91" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W91" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X91" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="92" spans="1:24" x14ac:dyDescent="0.3">
@@ -8997,13 +8997,13 @@
         <v>395</v>
       </c>
       <c r="V92" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W92" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X92" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="93" spans="1:24" x14ac:dyDescent="0.3">
@@ -9065,13 +9065,13 @@
         <v>399</v>
       </c>
       <c r="V93" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W93" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X93" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="94" spans="1:24" x14ac:dyDescent="0.3">
@@ -9133,13 +9133,13 @@
         <v>404</v>
       </c>
       <c r="V94" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W94" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X94" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="95" spans="1:24" x14ac:dyDescent="0.3">
@@ -9201,13 +9201,13 @@
         <v>409</v>
       </c>
       <c r="V95" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W95" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X95" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="96" spans="1:24" x14ac:dyDescent="0.3">
@@ -9269,13 +9269,13 @@
         <v>414</v>
       </c>
       <c r="V96" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W96" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X96" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="97" spans="1:24" x14ac:dyDescent="0.3">
@@ -9337,13 +9337,13 @@
         <v>419</v>
       </c>
       <c r="V97" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W97" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X97" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="98" spans="1:24" x14ac:dyDescent="0.3">
@@ -9405,13 +9405,13 @@
         <v>424</v>
       </c>
       <c r="V98" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W98" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X98" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="99" spans="1:24" x14ac:dyDescent="0.3">
@@ -9473,13 +9473,13 @@
         <v>29</v>
       </c>
       <c r="V99" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W99" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X99" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="100" spans="1:24" x14ac:dyDescent="0.3">
@@ -9541,13 +9541,13 @@
         <v>207</v>
       </c>
       <c r="V100" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W100" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X100" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="101" spans="1:24" x14ac:dyDescent="0.3">
@@ -9609,13 +9609,13 @@
         <v>433</v>
       </c>
       <c r="V101" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W101" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X101" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="102" spans="1:24" x14ac:dyDescent="0.3">
@@ -9677,13 +9677,13 @@
         <v>438</v>
       </c>
       <c r="V102" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W102" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X102" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="103" spans="1:24" x14ac:dyDescent="0.3">
@@ -9745,13 +9745,13 @@
         <v>444</v>
       </c>
       <c r="V103" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W103" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X103" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="104" spans="1:24" x14ac:dyDescent="0.3">
@@ -9810,13 +9810,13 @@
         <v>447</v>
       </c>
       <c r="V104" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W104" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X104" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="105" spans="1:24" x14ac:dyDescent="0.3">
@@ -9878,13 +9878,13 @@
         <v>29</v>
       </c>
       <c r="V105" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W105" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X105" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="106" spans="1:24" x14ac:dyDescent="0.3">
@@ -9946,13 +9946,13 @@
         <v>455</v>
       </c>
       <c r="V106" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W106" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X106" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="107" spans="1:24" x14ac:dyDescent="0.3">
@@ -10014,13 +10014,13 @@
         <v>29</v>
       </c>
       <c r="V107" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W107" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X107" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="108" spans="1:24" x14ac:dyDescent="0.3">
@@ -10082,13 +10082,13 @@
         <v>462</v>
       </c>
       <c r="V108" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W108" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X108" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="109" spans="1:24" x14ac:dyDescent="0.3">
@@ -10150,13 +10150,13 @@
         <v>466</v>
       </c>
       <c r="V109" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W109" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X109" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="110" spans="1:24" x14ac:dyDescent="0.3">
@@ -10218,13 +10218,13 @@
         <v>470</v>
       </c>
       <c r="V110" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W110" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X110" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="111" spans="1:24" x14ac:dyDescent="0.3">
@@ -10283,13 +10283,13 @@
         <v>472</v>
       </c>
       <c r="V111" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W111" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X111" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="112" spans="1:24" x14ac:dyDescent="0.3">
@@ -10351,13 +10351,13 @@
         <v>112</v>
       </c>
       <c r="V112" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W112" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X112" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="113" spans="1:24" x14ac:dyDescent="0.3">
@@ -10419,13 +10419,13 @@
         <v>426</v>
       </c>
       <c r="V113" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W113" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X113" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="114" spans="1:24" x14ac:dyDescent="0.3">
@@ -10484,13 +10484,13 @@
         <v>482</v>
       </c>
       <c r="V114" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W114" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X114" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="115" spans="1:24" x14ac:dyDescent="0.3">
@@ -10552,13 +10552,13 @@
         <v>487</v>
       </c>
       <c r="V115" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W115" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X115" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="116" spans="1:24" x14ac:dyDescent="0.3">
@@ -10620,13 +10620,13 @@
         <v>492</v>
       </c>
       <c r="V116" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W116" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X116" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="117" spans="1:24" x14ac:dyDescent="0.3">
@@ -10688,13 +10688,13 @@
         <v>29</v>
       </c>
       <c r="V117" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W117" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X117" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="118" spans="1:24" x14ac:dyDescent="0.3">
@@ -10756,13 +10756,13 @@
         <v>29</v>
       </c>
       <c r="V118" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W118" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X118" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="119" spans="1:24" x14ac:dyDescent="0.3">
@@ -10821,13 +10821,13 @@
         <v>500</v>
       </c>
       <c r="V119" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W119" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X119" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="120" spans="1:24" x14ac:dyDescent="0.3">
@@ -10889,13 +10889,13 @@
         <v>318</v>
       </c>
       <c r="V120" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W120" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X120" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="121" spans="1:24" x14ac:dyDescent="0.3">
@@ -10954,13 +10954,13 @@
         <v>509</v>
       </c>
       <c r="V121" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W121" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X121" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="122" spans="1:24" x14ac:dyDescent="0.3">
@@ -11022,13 +11022,13 @@
         <v>53</v>
       </c>
       <c r="V122" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W122" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X122" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="123" spans="1:24" x14ac:dyDescent="0.3">
@@ -11090,13 +11090,13 @@
         <v>318</v>
       </c>
       <c r="V123" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W123" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X123" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="124" spans="1:24" x14ac:dyDescent="0.3">
@@ -11158,13 +11158,13 @@
         <v>462</v>
       </c>
       <c r="V124" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W124" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X124" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="125" spans="1:24" x14ac:dyDescent="0.3">
@@ -11226,13 +11226,13 @@
         <v>462</v>
       </c>
       <c r="V125" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W125" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X125" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="126" spans="1:24" x14ac:dyDescent="0.3">
@@ -11294,13 +11294,13 @@
         <v>318</v>
       </c>
       <c r="V126" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W126" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X126" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="127" spans="1:24" x14ac:dyDescent="0.3">
@@ -11362,13 +11362,13 @@
         <v>527</v>
       </c>
       <c r="V127" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W127" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X127" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="128" spans="1:24" x14ac:dyDescent="0.3">
@@ -11430,13 +11430,13 @@
         <v>531</v>
       </c>
       <c r="V128" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W128" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X128" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="129" spans="1:24" x14ac:dyDescent="0.3">
@@ -11498,13 +11498,13 @@
         <v>535</v>
       </c>
       <c r="V129" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W129" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X129" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="130" spans="1:24" x14ac:dyDescent="0.3">
@@ -11566,13 +11566,13 @@
         <v>541</v>
       </c>
       <c r="V130" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W130" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X130" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="131" spans="1:24" x14ac:dyDescent="0.3">
@@ -11631,13 +11631,13 @@
         <v>543</v>
       </c>
       <c r="V131" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W131" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X131" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="132" spans="1:24" x14ac:dyDescent="0.3">
@@ -11699,13 +11699,13 @@
         <v>318</v>
       </c>
       <c r="V132" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W132" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X132" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="133" spans="1:24" x14ac:dyDescent="0.3">
@@ -11767,13 +11767,13 @@
         <v>552</v>
       </c>
       <c r="V133" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W133" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X133" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="134" spans="1:24" x14ac:dyDescent="0.3">
@@ -11835,13 +11835,13 @@
         <v>29</v>
       </c>
       <c r="V134" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W134" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X134" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="135" spans="1:24" x14ac:dyDescent="0.3">
@@ -11903,13 +11903,13 @@
         <v>318</v>
       </c>
       <c r="V135" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W135" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X135" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="136" spans="1:24" x14ac:dyDescent="0.3">
@@ -11974,13 +11974,13 @@
         <v>563</v>
       </c>
       <c r="V136" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W136" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X136" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="137" spans="1:24" x14ac:dyDescent="0.3">
@@ -12039,13 +12039,13 @@
         <v>566</v>
       </c>
       <c r="V137" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W137" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X137" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="138" spans="1:24" x14ac:dyDescent="0.3">
@@ -12107,13 +12107,13 @@
         <v>570</v>
       </c>
       <c r="V138" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W138" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X138" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="139" spans="1:24" x14ac:dyDescent="0.3">
@@ -12175,13 +12175,13 @@
         <v>574</v>
       </c>
       <c r="V139" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W139" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X139" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="140" spans="1:24" x14ac:dyDescent="0.3">
@@ -12246,13 +12246,13 @@
         <v>578</v>
       </c>
       <c r="V140" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W140" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X140" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="141" spans="1:24" x14ac:dyDescent="0.3">
@@ -12314,13 +12314,13 @@
         <v>583</v>
       </c>
       <c r="V141" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W141" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X141" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="142" spans="1:24" x14ac:dyDescent="0.3">
@@ -12382,13 +12382,13 @@
         <v>492</v>
       </c>
       <c r="V142" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W142" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X142" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="143" spans="1:24" x14ac:dyDescent="0.3">
@@ -12450,13 +12450,13 @@
         <v>588</v>
       </c>
       <c r="V143" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W143" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X143" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="144" spans="1:24" x14ac:dyDescent="0.3">
@@ -12518,13 +12518,13 @@
         <v>593</v>
       </c>
       <c r="V144" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W144" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X144" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="145" spans="1:24" x14ac:dyDescent="0.3">
@@ -12583,13 +12583,13 @@
         <v>596</v>
       </c>
       <c r="V145" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W145" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X145" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="146" spans="1:24" x14ac:dyDescent="0.3">
@@ -12651,13 +12651,13 @@
         <v>600</v>
       </c>
       <c r="V146" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W146" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X146" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="147" spans="1:24" x14ac:dyDescent="0.3">
@@ -12719,13 +12719,13 @@
         <v>605</v>
       </c>
       <c r="V147" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W147" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X147" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="148" spans="1:24" x14ac:dyDescent="0.3">
@@ -12787,13 +12787,13 @@
         <v>607</v>
       </c>
       <c r="V148" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W148" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X148" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="149" spans="1:24" x14ac:dyDescent="0.3">
@@ -12855,13 +12855,13 @@
         <v>367</v>
       </c>
       <c r="V149" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W149" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X149" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="150" spans="1:24" x14ac:dyDescent="0.3">
@@ -12923,13 +12923,13 @@
         <v>614</v>
       </c>
       <c r="V150" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W150" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X150" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="151" spans="1:24" x14ac:dyDescent="0.3">
@@ -12991,13 +12991,13 @@
         <v>574</v>
       </c>
       <c r="V151" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W151" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X151" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="152" spans="1:24" x14ac:dyDescent="0.3">
@@ -13059,13 +13059,13 @@
         <v>621</v>
       </c>
       <c r="V152" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W152" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X152" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="153" spans="1:24" x14ac:dyDescent="0.3">
@@ -13127,13 +13127,13 @@
         <v>624</v>
       </c>
       <c r="V153" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W153" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X153" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="154" spans="1:24" x14ac:dyDescent="0.3">
@@ -13195,13 +13195,13 @@
         <v>629</v>
       </c>
       <c r="V154" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W154" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X154" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="155" spans="1:24" x14ac:dyDescent="0.3">
@@ -13263,13 +13263,13 @@
         <v>29</v>
       </c>
       <c r="V155" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W155" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X155" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="156" spans="1:24" x14ac:dyDescent="0.3">
@@ -13331,13 +13331,13 @@
         <v>638</v>
       </c>
       <c r="V156" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W156" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X156" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="157" spans="1:24" x14ac:dyDescent="0.3">
@@ -13399,13 +13399,13 @@
         <v>642</v>
       </c>
       <c r="V157" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W157" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X157" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="158" spans="1:24" x14ac:dyDescent="0.3">
@@ -13467,13 +13467,13 @@
         <v>647</v>
       </c>
       <c r="V158" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W158" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X158" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="159" spans="1:24" x14ac:dyDescent="0.3">
@@ -13535,13 +13535,13 @@
         <v>318</v>
       </c>
       <c r="V159" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W159" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X159" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="160" spans="1:24" x14ac:dyDescent="0.3">
@@ -13603,13 +13603,13 @@
         <v>654</v>
       </c>
       <c r="V160" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W160" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X160" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="161" spans="1:24" x14ac:dyDescent="0.3">
@@ -13671,13 +13671,13 @@
         <v>657</v>
       </c>
       <c r="V161" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W161" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X161" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="162" spans="1:24" x14ac:dyDescent="0.3">
@@ -13739,13 +13739,13 @@
         <v>29</v>
       </c>
       <c r="V162" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W162" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X162" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="163" spans="1:24" x14ac:dyDescent="0.3">
@@ -13807,13 +13807,13 @@
         <v>665</v>
       </c>
       <c r="V163" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W163" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X163" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="164" spans="1:24" x14ac:dyDescent="0.3">
@@ -13875,13 +13875,13 @@
         <v>669</v>
       </c>
       <c r="V164" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W164" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X164" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="165" spans="1:24" x14ac:dyDescent="0.3">
@@ -13943,13 +13943,13 @@
         <v>672</v>
       </c>
       <c r="V165" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W165" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X165" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="166" spans="1:24" x14ac:dyDescent="0.3">
@@ -14011,13 +14011,13 @@
         <v>676</v>
       </c>
       <c r="V166" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W166" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X166" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="167" spans="1:24" x14ac:dyDescent="0.3">
@@ -14082,13 +14082,13 @@
         <v>680</v>
       </c>
       <c r="V167" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W167" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X167" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="168" spans="1:24" x14ac:dyDescent="0.3">
@@ -14147,13 +14147,13 @@
         <v>682</v>
       </c>
       <c r="V168" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W168" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X168" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="169" spans="1:24" x14ac:dyDescent="0.3">
@@ -14212,13 +14212,13 @@
         <v>684</v>
       </c>
       <c r="V169" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W169" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X169" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="170" spans="1:24" x14ac:dyDescent="0.3">
@@ -14277,13 +14277,13 @@
         <v>686</v>
       </c>
       <c r="V170" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W170" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X170" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="171" spans="1:24" x14ac:dyDescent="0.3">
@@ -14342,13 +14342,13 @@
         <v>688</v>
       </c>
       <c r="V171" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W171" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X171" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="172" spans="1:24" x14ac:dyDescent="0.3">
@@ -14410,13 +14410,13 @@
         <v>29</v>
       </c>
       <c r="V172" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W172" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X172" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="173" spans="1:24" x14ac:dyDescent="0.3">
@@ -14478,13 +14478,13 @@
         <v>578</v>
       </c>
       <c r="V173" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W173" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X173" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="174" spans="1:24" x14ac:dyDescent="0.3">
@@ -14546,13 +14546,13 @@
         <v>694</v>
       </c>
       <c r="V174" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W174" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X174" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="175" spans="1:24" x14ac:dyDescent="0.3">
@@ -14614,13 +14614,13 @@
         <v>697</v>
       </c>
       <c r="V175" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W175" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X175" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="176" spans="1:24" x14ac:dyDescent="0.3">
@@ -14679,13 +14679,13 @@
         <v>700</v>
       </c>
       <c r="V176" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W176" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X176" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="177" spans="1:24" x14ac:dyDescent="0.3">
@@ -14747,13 +14747,13 @@
         <v>703</v>
       </c>
       <c r="V177" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W177" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X177" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="178" spans="1:24" x14ac:dyDescent="0.3">
@@ -14815,13 +14815,13 @@
         <v>707</v>
       </c>
       <c r="V178" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W178" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X178" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="179" spans="1:24" x14ac:dyDescent="0.3">
@@ -14883,13 +14883,13 @@
         <v>712</v>
       </c>
       <c r="V179" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W179" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X179" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="180" spans="1:24" x14ac:dyDescent="0.3">
@@ -14954,13 +14954,13 @@
         <v>717</v>
       </c>
       <c r="V180" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W180" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X180" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="181" spans="1:24" x14ac:dyDescent="0.3">
@@ -15025,13 +15025,13 @@
         <v>723</v>
       </c>
       <c r="V181" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W181" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X181" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="182" spans="1:24" x14ac:dyDescent="0.3">
@@ -15093,13 +15093,13 @@
         <v>727</v>
       </c>
       <c r="V182" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W182" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X182" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="183" spans="1:24" x14ac:dyDescent="0.3">
@@ -15164,13 +15164,13 @@
         <v>733</v>
       </c>
       <c r="V183" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W183" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X183" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="184" spans="1:24" x14ac:dyDescent="0.3">
@@ -15235,13 +15235,13 @@
         <v>29</v>
       </c>
       <c r="V184" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W184" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X184" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="185" spans="1:24" x14ac:dyDescent="0.3">
@@ -15306,13 +15306,13 @@
         <v>743</v>
       </c>
       <c r="V185" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W185" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X185" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="186" spans="1:24" x14ac:dyDescent="0.3">
@@ -15377,13 +15377,13 @@
         <v>748</v>
       </c>
       <c r="V186" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W186" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X186" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="187" spans="1:24" x14ac:dyDescent="0.3">
@@ -15451,13 +15451,13 @@
         <v>29</v>
       </c>
       <c r="V187" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W187" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X187" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="188" spans="1:24" x14ac:dyDescent="0.3">
@@ -15519,13 +15519,13 @@
         <v>757</v>
       </c>
       <c r="V188" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W188" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X188" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="189" spans="1:24" x14ac:dyDescent="0.3">
@@ -15590,13 +15590,13 @@
         <v>29</v>
       </c>
       <c r="V189" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="W189" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="X189" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>